<commit_message>
add gemini 2.5 pro
</commit_message>
<xml_diff>
--- a/results_summary_gemini.xlsx
+++ b/results_summary_gemini.xlsx
@@ -1,41 +1,131 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minhe\python\AI_research\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4940C4-5E3E-434F-8ECD-A3D916C9421A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="gemini-2.5-pro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>CoT</t>
-  </si>
-  <si>
-    <t>2022_12A</t>
-  </si>
-  <si>
-    <t>2022_12B</t>
-  </si>
-  <si>
-    <t>benchmark</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
+  <si>
+    <t>Problem 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5/5</t>
+  </si>
+  <si>
+    <t>Problem 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2/5</t>
+  </si>
+  <si>
+    <t>Problem 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3/5</t>
+  </si>
+  <si>
+    <t>Problem 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4/5</t>
+  </si>
+  <si>
+    <t>Problem 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0/5</t>
+  </si>
+  <si>
+    <t>Problem 6</t>
+  </si>
+  <si>
+    <t>Problem 7</t>
+  </si>
+  <si>
+    <t>Problem 8</t>
+  </si>
+  <si>
+    <t>Problem 9</t>
+  </si>
+  <si>
+    <t>Problem 10</t>
+  </si>
+  <si>
+    <t>Problem 11</t>
+  </si>
+  <si>
+    <t>Problem 12</t>
+  </si>
+  <si>
+    <t>Problem 13</t>
+  </si>
+  <si>
+    <t>Problem 14</t>
+  </si>
+  <si>
+    <t>Problem 15</t>
+  </si>
+  <si>
+    <t>Problem 16</t>
+  </si>
+  <si>
+    <t>Problem 17</t>
+  </si>
+  <si>
+    <t>Problem 18</t>
+  </si>
+  <si>
+    <t>Problem 19</t>
+  </si>
+  <si>
+    <t>Problem 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/5</t>
+  </si>
+  <si>
+    <t>Problem 21</t>
+  </si>
+  <si>
+    <t>Problem 22</t>
+  </si>
+  <si>
+    <t>Problem 23</t>
+  </si>
+  <si>
+    <t>Problem 24</t>
+  </si>
+  <si>
+    <t>Problem 25</t>
+  </si>
+  <si>
+    <t>2022 12A</t>
+  </si>
+  <si>
+    <t>2022 12B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,15 +142,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -83,28 +179,182 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -142,7 +392,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -176,6 +426,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -210,9 +461,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -385,30 +637,297 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="13"/>
+      <c r="B1" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="C3" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
+      <c r="B4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 2024 12B for gemini pro 2.5
</commit_message>
<xml_diff>
--- a/results_summary_gemini.xlsx
+++ b/results_summary_gemini.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minhe\python\AI_research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4940C4-5E3E-434F-8ECD-A3D916C9421A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CC3C01-45E3-464D-A29D-9AF1F97AFD00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="34">
   <si>
     <t>Problem 1</t>
   </si>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>2022 12B</t>
+  </si>
+  <si>
+    <t>2024 12B</t>
   </si>
 </sst>
 </file>
@@ -156,7 +159,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -255,13 +258,65 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -274,7 +329,9 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -287,7 +344,9 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -297,16 +356,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -321,19 +374,25 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -638,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -646,289 +705,497 @@
     <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="8"/>
       <c r="B1" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="D1" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="D3" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="D4" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="D5" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="D6" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="D7" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="D8" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="D9" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="D10" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="D11" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="D12" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="D13" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="D14" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="D15" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="D16" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="D17" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="D18" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="D19" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="D20" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="D21" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="D22" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="D23" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+      <c r="D24" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="D25" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="6" t="s">
         <v>3</v>
       </c>
+      <c r="D26" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>